<commit_message>
remove null values in the answer table and replace them with "not answered"
</commit_message>
<xml_diff>
--- a/Source/codebook_DigiLearnHF_2025-09-11_12-21.xlsx
+++ b/Source/codebook_DigiLearnHF_2025-09-11_12-21.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tehranim.TIB.001\Desktop\Computer-20260504T112359Z-3-001\Computer\Master Thesis\EER-Questionaries\kg_corrected_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tehranim.TIB.001\Desktop\Computer-20260504T112359Z-3-001\Computer\Master Thesis\EER-Questionaries\Questionnarie-KG\Source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92EA7777-ECBE-4206-8BFD-018029C1CA1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B06734-A109-4DD1-90C7-D068E40A88C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="212" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="212" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DigiLearnHF" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">queszionnaire!$A$1:$A$240</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="236">
   <si>
     <t>Variable</t>
   </si>
@@ -723,9 +723,6 @@
   </si>
   <si>
     <t>User_Id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   </t>
   </si>
   <si>
     <t xml:space="preserve">          </t>
@@ -1246,7 +1243,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>11</v>
@@ -1266,7 +1263,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>11</v>
@@ -1286,7 +1283,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>11</v>
@@ -1306,7 +1303,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>11</v>
@@ -1326,7 +1323,7 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>11</v>
@@ -1346,7 +1343,7 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>11</v>
@@ -1366,7 +1363,7 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>11</v>
@@ -1386,7 +1383,7 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>11</v>
@@ -1466,7 +1463,7 @@
         <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>11</v>
@@ -1486,7 +1483,7 @@
         <v>3</v>
       </c>
       <c r="D15" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>11</v>
@@ -1506,7 +1503,7 @@
         <v>4</v>
       </c>
       <c r="D16" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>11</v>
@@ -1526,7 +1523,7 @@
         <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>11</v>
@@ -1546,7 +1543,7 @@
         <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>11</v>
@@ -1566,7 +1563,7 @@
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>11</v>
@@ -1586,7 +1583,7 @@
         <v>8</v>
       </c>
       <c r="D20" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>11</v>
@@ -1606,7 +1603,7 @@
         <v>9</v>
       </c>
       <c r="D21" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>11</v>
@@ -1686,7 +1683,7 @@
         <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>11</v>
@@ -1706,7 +1703,7 @@
         <v>3</v>
       </c>
       <c r="D26" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>11</v>
@@ -1726,7 +1723,7 @@
         <v>4</v>
       </c>
       <c r="D27" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>11</v>
@@ -1746,7 +1743,7 @@
         <v>5</v>
       </c>
       <c r="D28" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>11</v>
@@ -1766,7 +1763,7 @@
         <v>6</v>
       </c>
       <c r="D29" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>11</v>
@@ -1786,7 +1783,7 @@
         <v>7</v>
       </c>
       <c r="D30" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>11</v>
@@ -1806,7 +1803,7 @@
         <v>8</v>
       </c>
       <c r="D31" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>11</v>
@@ -1826,7 +1823,7 @@
         <v>9</v>
       </c>
       <c r="D32" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>11</v>
@@ -1986,7 +1983,7 @@
         <v>2</v>
       </c>
       <c r="D40" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>11</v>
@@ -2006,7 +2003,7 @@
         <v>3</v>
       </c>
       <c r="D41" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>11</v>
@@ -2026,7 +2023,7 @@
         <v>4</v>
       </c>
       <c r="D42" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>11</v>
@@ -2046,7 +2043,7 @@
         <v>5</v>
       </c>
       <c r="D43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>11</v>
@@ -2066,7 +2063,7 @@
         <v>6</v>
       </c>
       <c r="D44" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>11</v>
@@ -2086,7 +2083,7 @@
         <v>7</v>
       </c>
       <c r="D45" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>11</v>
@@ -2106,7 +2103,7 @@
         <v>8</v>
       </c>
       <c r="D46" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>11</v>
@@ -2126,7 +2123,7 @@
         <v>9</v>
       </c>
       <c r="D47" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>11</v>
@@ -2238,7 +2235,7 @@
         <v>2</v>
       </c>
       <c r="D53" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>11</v>
@@ -2258,7 +2255,7 @@
         <v>3</v>
       </c>
       <c r="D54" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>11</v>
@@ -2278,7 +2275,7 @@
         <v>4</v>
       </c>
       <c r="D55" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>11</v>
@@ -2298,7 +2295,7 @@
         <v>5</v>
       </c>
       <c r="D56" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>11</v>
@@ -2318,7 +2315,7 @@
         <v>6</v>
       </c>
       <c r="D57" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>11</v>
@@ -2338,7 +2335,7 @@
         <v>7</v>
       </c>
       <c r="D58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>11</v>
@@ -2358,7 +2355,7 @@
         <v>8</v>
       </c>
       <c r="D59" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>11</v>
@@ -2378,7 +2375,7 @@
         <v>9</v>
       </c>
       <c r="D60" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>11</v>
@@ -3029,7 +3026,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
-        <v>226</v>
+        <v>59</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>60</v>
@@ -3487,7 +3484,7 @@
         <v>12</v>
       </c>
       <c r="I115" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
@@ -6292,7 +6289,7 @@
         <v>161</v>
       </c>
       <c r="C34" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>